<commit_message>
sprint 6 started and all developer stable files created
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,11 +477,6 @@
           <t>capital_allocation_label</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>capital_allocation_pattern</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -526,7 +521,6 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -571,7 +565,6 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -616,7 +609,6 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -661,7 +653,6 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -707,7 +698,6 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -752,7 +742,6 @@
           <t>Liquidating Assets</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -797,7 +786,6 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -843,7 +831,6 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -889,22 +876,21 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ATGL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Axis Bank Ltd</t>
+          <t>Adani Total Gas Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -919,9 +905,7 @@
           <t>Insufficient Data</t>
         </is>
       </c>
-      <c r="H11" t="n">
-        <v>14.74</v>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="b">
         <v>0</v>
@@ -931,25 +915,24 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bajaj Auto Ltd</t>
+          <t>Axis Bank Ltd</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -965,7 +948,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>8.130000000000001</v>
+        <v>14.74</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="b">
@@ -976,25 +959,24 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bajaj Finserv Ltd</t>
+          <t>Bajaj Auto Ltd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -1010,7 +992,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>20.97</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
@@ -1021,20 +1003,19 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BAJAJHLDNG</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bajaj Holdings &amp; Investment Ltd</t>
+          <t>Bajaj Finserv Ltd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1055,7 +1036,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>31.61</v>
+        <v>20.97</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
@@ -1066,20 +1047,19 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>BAJAJHLDNG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bajaj Finance Ltd</t>
+          <t>Bajaj Holdings &amp; Investment Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1100,7 +1080,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>24.35</v>
+        <v>31.61</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="b">
@@ -1111,20 +1091,19 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BANKBARODA</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bank of Baroda</t>
+          <t>Bajaj Finance Ltd</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1145,7 +1124,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>17.48</v>
+        <v>24.35</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="b">
@@ -1159,22 +1138,21 @@
           <t>Growth Funded by Debt</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>BANKBARODA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bharat Electronics Ltd</t>
+          <t>Bank of Baroda</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -1190,7 +1168,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>10.75</v>
+        <v>17.48</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="b">
@@ -1201,25 +1179,24 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bharti Airtel Ltd</t>
+          <t>Bharat Electronics Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1235,7 +1212,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>13.17</v>
+        <v>10.75</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="b">
@@ -1249,68 +1226,66 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Bharti Airtel Ltd</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>13.17</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>BHEL</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t xml:space="preserve">Bharat Heavy Electricals Limited
 </t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>-4.73</v>
-      </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="b">
-        <v>0</v>
-      </c>
-      <c r="K19" t="b">
-        <v>0</v>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Distress Signal</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BOSCHLTD</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Bosch Ltd</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1326,7 +1301,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>6.72</v>
+        <v>-4.73</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="b">
@@ -1337,25 +1312,24 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation Ltd</t>
+          <t>Bosch Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -1371,7 +1345,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>8.48</v>
+        <v>6.72</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="b">
@@ -1382,25 +1356,24 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Britannia Industries Ltd</t>
+          <t>Bharat Petroleum Corporation Ltd</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1416,7 +1389,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>8.69</v>
+        <v>8.48</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="b">
@@ -1427,25 +1400,24 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CANBK</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Canara Bank</t>
+          <t>Britannia Industries Ltd</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1461,7 +1433,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>18.18</v>
+        <v>8.69</v>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="b">
@@ -1472,20 +1444,19 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CHOLAFIN</t>
+          <t>CANBK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
+          <t>Canara Bank</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1506,7 +1477,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>21.94</v>
+        <v>18.18</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="b">
@@ -1517,71 +1488,69 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cholamandalam Investment &amp; Finance Company Ltd</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>21.94</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" t="b">
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>CIPLA</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t xml:space="preserve">Cipla Ltd
 </t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>9.51</v>
-      </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="b">
-        <v>0</v>
-      </c>
-      <c r="K25" t="b">
-        <v>0</v>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>COALINDIA</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Coal India Ltd</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Materials</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1597,7 +1566,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>7.4</v>
+        <v>9.51</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="b">
@@ -1611,22 +1580,21 @@
           <t>Reinvestor</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DABUR</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dabur India Ltd</t>
+          <t>Coal India Ltd</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -1642,7 +1610,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>7.81</v>
+        <v>7.4</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="b">
@@ -1653,25 +1621,24 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DIVISLAB</t>
+          <t>DABUR</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Divis Laboratories Ltd</t>
+          <t>Dabur India Ltd</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1687,7 +1654,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>9.66</v>
+        <v>7.81</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="b">
@@ -1698,25 +1665,24 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DLF</t>
+          <t>DIVISLAB</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DLF Ltd</t>
+          <t>Divis Laboratories Ltd</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -1732,7 +1698,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>-5.14</v>
+        <v>9.66</v>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="b">
@@ -1743,25 +1709,24 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>DLF</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Avenue Supermarts Ltd</t>
+          <t>DLF Ltd</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -1777,7 +1742,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>20.48</v>
+        <v>-5.14</v>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="b">
@@ -1788,25 +1753,24 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>DMART</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dr Reddys Laboratories Ltd</t>
+          <t>Avenue Supermarts Ltd</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -1822,7 +1786,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>12.64</v>
+        <v>20.48</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="b">
@@ -1833,25 +1797,24 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Eicher Motors Ltd</t>
+          <t>Dr Reddys Laboratories Ltd</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1867,7 +1830,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>11.04</v>
+        <v>12.64</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="b">
@@ -1881,22 +1844,21 @@
           <t>Reinvestor</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GAIL (India) Ltd</t>
+          <t>Eicher Motors Ltd</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1912,7 +1874,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>11.83</v>
+        <v>11.04</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="b">
@@ -1923,25 +1885,24 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GODREJCP</t>
+          <t>GAIL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Godrej Consumer Products Ltd</t>
+          <t>GAIL (India) Ltd</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1957,7 +1918,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>6.45</v>
+        <v>11.83</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="b">
@@ -1968,25 +1929,24 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>GODREJCP</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Grasim Industries Ltd</t>
+          <t>Godrej Consumer Products Ltd</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -2002,7 +1962,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>11.15</v>
+        <v>6.45</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="b">
@@ -2013,20 +1973,19 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hindustan Aeronautics Ltd</t>
+          <t>Grasim Industries Ltd</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2047,7 +2006,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>8.710000000000001</v>
+        <v>11.15</v>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="b">
@@ -2058,20 +2017,19 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>HAVELLS</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Havells India Ltd</t>
+          <t>Hindustan Aeronautics Ltd</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2092,7 +2050,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>13.04</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="b">
@@ -2106,22 +2064,21 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>HAVELLS</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HCL Technologies Ltd</t>
+          <t>Havells India Ltd</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2137,7 +2094,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>12.71</v>
+        <v>13.04</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="b">
@@ -2151,22 +2108,21 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HDFC Bank Ltd</t>
+          <t>HCL Technologies Ltd</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2182,7 +2138,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>21.95</v>
+        <v>12.71</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="b">
@@ -2193,20 +2149,19 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HDFC Life Insurance Company Ltd</t>
+          <t>HDFC Bank Ltd</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2227,7 +2182,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>21.17</v>
+        <v>21.95</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="b">
@@ -2238,71 +2193,69 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr"/>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HDFC Life Insurance Company Ltd</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>21.17</v>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="b">
+        <v>0</v>
+      </c>
+      <c r="K41" t="b">
+        <v>0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>HEROMOTOCO</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t xml:space="preserve">Hero MotoCorp Ltd
 </t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="b">
-        <v>0</v>
-      </c>
-      <c r="K41" t="b">
-        <v>0</v>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>HINDALCO</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Hindalco Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Materials</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -2318,7 +2271,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>10.59</v>
+        <v>2.15</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="b">
@@ -2332,68 +2285,66 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Hindalco Industries Ltd</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="b">
+        <v>0</v>
+      </c>
+      <c r="K43" t="b">
+        <v>0</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>HINDUNILVR</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t xml:space="preserve">Hindustan Unilever Ltd
 </t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="b">
-        <v>0</v>
-      </c>
-      <c r="K43" t="b">
-        <v>0</v>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ICICIBANK</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>ICICI Bank Ltd</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Financials</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2409,7 +2360,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>17.25</v>
+        <v>9.5</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="b">
@@ -2420,20 +2371,19 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ICICI Lombard General Insurance Company Ltd</t>
+          <t>ICICI Bank Ltd</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2454,7 +2404,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>12.91</v>
+        <v>17.25</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="b">
@@ -2465,20 +2415,19 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ICICIPRULI</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ICICI Prudential Life Insurance Company Ltd</t>
+          <t>ICICI Lombard General Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2499,7 +2448,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>16.85</v>
+        <v>12.91</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="b">
@@ -2510,25 +2459,24 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>ICICIPRULI</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Interglobe Aviation Ltd</t>
+          <t>ICICI Prudential Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -2544,7 +2492,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>19.31</v>
+        <v>16.85</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="b">
@@ -2555,25 +2503,24 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IndusInd Bank Ltd</t>
+          <t>Interglobe Aviation Ltd</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -2589,7 +2536,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>15.5</v>
+        <v>19.31</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="b">
@@ -2600,25 +2547,24 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Pre-Revenue</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>INDUSINDBK</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Infosys Ltd</t>
+          <t>IndusInd Bank Ltd</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -2634,7 +2580,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>13.2</v>
+        <v>15.5</v>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="b">
@@ -2645,71 +2591,69 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr"/>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Infosys Ltd</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="b">
+        <v>0</v>
+      </c>
+      <c r="K50" t="b">
+        <v>0</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>IOC</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t xml:space="preserve">Indian Oil Corporation
 </t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Energy</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H50" t="n">
-        <v>8.01</v>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="b">
-        <v>0</v>
-      </c>
-      <c r="K50" t="b">
-        <v>0</v>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>IRCTC</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -2725,7 +2669,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>17.96</v>
+        <v>8.01</v>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="b">
@@ -2736,25 +2680,24 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IRFC</t>
+          <t>IRCTC</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Indian Railway Finance Corporation Ltd</t>
+          <t>Indian Railway Catering &amp; Tourism Corporation Ltd</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -2770,7 +2713,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>19.07</v>
+        <v>17.96</v>
       </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="b">
@@ -2781,71 +2724,69 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Indian Railway Finance Corporation Ltd</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>19.07</v>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="b">
+        <v>0</v>
+      </c>
+      <c r="K53" t="b">
+        <v>0</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>ITC</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t xml:space="preserve">ITC Ltd
 </t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>7.95</v>
-      </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="b">
-        <v>0</v>
-      </c>
-      <c r="K53" t="b">
-        <v>0</v>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>JINDALSTEL</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Jindal Steel &amp; Power Ltd</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Materials</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -2861,7 +2802,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>1.4</v>
+        <v>7.95</v>
       </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="b">
@@ -2872,25 +2813,24 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr"/>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Jio Financial Services Ltd</t>
+          <t>Jindal Steel &amp; Power Ltd</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2905,7 +2845,9 @@
           <t>Insufficient Data</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>1.4</v>
+      </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="b">
         <v>0</v>
@@ -2918,22 +2860,21 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>JSW Energy Ltd</t>
+          <t>Jio Financial Services Ltd</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -2948,9 +2889,7 @@
           <t>Insufficient Data</t>
         </is>
       </c>
-      <c r="H56" t="n">
-        <v>4.68</v>
-      </c>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="b">
         <v>0</v>
@@ -2963,22 +2902,21 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>JSWENERGY</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>JSW Steel Ltd</t>
+          <t>JSW Energy Ltd</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -2994,7 +2932,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>15.6</v>
+        <v>4.68</v>
       </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="b">
@@ -3005,68 +2943,66 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>JSW Steel Ltd</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="b">
+        <v>0</v>
+      </c>
+      <c r="K58" t="b">
+        <v>0</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>KOTAKBANK</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t xml:space="preserve">Kotak Mahindra Bank Ltd
 </t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H58" t="n">
-        <v>13.52</v>
-      </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="b">
-        <v>0</v>
-      </c>
-      <c r="K58" t="b">
-        <v>0</v>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>LICI</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Life Insurance Corporation of India</t>
-        </is>
-      </c>
       <c r="C59" t="inlineStr">
         <is>
           <t>Financials</t>
@@ -3085,7 +3021,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>8.16</v>
+        <v>13.52</v>
       </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="b">
@@ -3096,25 +3032,24 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LODHA</t>
+          <t>LICI</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Macrotech Developers Ltd</t>
+          <t>Life Insurance Corporation of India</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -3130,7 +3065,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>-2.83</v>
+        <v>8.16</v>
       </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="b">
@@ -3141,25 +3076,24 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>LODHA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro Ltd</t>
+          <t>Macrotech Developers Ltd</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -3175,7 +3109,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>10.34</v>
+        <v>-2.83</v>
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="b">
@@ -3186,25 +3120,24 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>LTIMindtree Ltd</t>
+          <t>Larsen &amp; Toubro Ltd</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -3220,7 +3153,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>30.33</v>
+        <v>10.34</v>
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="b">
@@ -3231,68 +3164,66 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr"/>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>LTIM</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>LTIMindtree Ltd</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>30.33</v>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="b">
+        <v>0</v>
+      </c>
+      <c r="K63" t="b">
+        <v>0</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>M&amp;M</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t xml:space="preserve">Mahindra &amp; Mahindra Ltd
 </t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H63" t="n">
-        <v>5.84</v>
-      </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="b">
-        <v>0</v>
-      </c>
-      <c r="K63" t="b">
-        <v>0</v>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>MARUTI</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Maruti Suzuki India Ltd</t>
-        </is>
-      </c>
       <c r="C64" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -3311,7 +3242,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>10.51</v>
+        <v>5.84</v>
       </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="b">
@@ -3322,20 +3253,19 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Samvardhana Motherson International Ltd</t>
+          <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3356,7 +3286,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>9.210000000000001</v>
+        <v>10.51</v>
       </c>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="b">
@@ -3367,25 +3297,24 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>NAUKRI</t>
+          <t>MOTHERSON</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Info Edge (India) Ltd</t>
+          <t>Samvardhana Motherson International Ltd</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -3401,7 +3330,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>17.12</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="b">
@@ -3415,22 +3344,21 @@
           <t>Mixed</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>NAUKRI</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Nestle India Ltd</t>
+          <t>Info Edge (India) Ltd</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -3446,7 +3374,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>14.55</v>
+        <v>17.12</v>
       </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="b">
@@ -3457,68 +3385,66 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr"/>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Nestle India Ltd</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="b">
+        <v>0</v>
+      </c>
+      <c r="K68" t="b">
+        <v>0</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>NHPC</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t xml:space="preserve">NHPC Ltd
 </t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H68" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="b">
-        <v>0</v>
-      </c>
-      <c r="K68" t="b">
-        <v>0</v>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>NTPC Ltd</t>
-        </is>
-      </c>
       <c r="C69" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -3537,7 +3463,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>12.22</v>
+        <v>1.4</v>
       </c>
       <c r="I69" t="inlineStr"/>
       <c r="J69" t="b">
@@ -3551,17 +3477,16 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Oil &amp; Natural Gas Corpn Ltd</t>
+          <t>NTPC Ltd</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3582,7 +3507,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>7</v>
+        <v>12.22</v>
       </c>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="b">
@@ -3596,22 +3521,21 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>PFC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Power Finance Corporation Ltd</t>
+          <t>Oil &amp; Natural Gas Corpn Ltd</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -3627,7 +3551,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>11.08</v>
+        <v>7</v>
       </c>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="b">
@@ -3638,25 +3562,24 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PIDILITIND</t>
+          <t>PFC</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Pidilite Industries Ltd</t>
+          <t>Power Finance Corporation Ltd</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -3672,7 +3595,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>11.84</v>
+        <v>11.08</v>
       </c>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="b">
@@ -3683,25 +3606,24 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PNB</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Punjab National Bank</t>
+          <t>Pidilite Industries Ltd</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -3717,7 +3639,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>15.9</v>
+        <v>11.84</v>
       </c>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="b">
@@ -3728,25 +3650,24 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>PNB</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Power Grid Corporation of India Ltd</t>
+          <t>Punjab National Bank</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -3762,7 +3683,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>5.51</v>
+        <v>15.9</v>
       </c>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="b">
@@ -3773,25 +3694,24 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>REC Ltd</t>
+          <t>Power Grid Corporation of India Ltd</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -3807,7 +3727,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>13.34</v>
+        <v>5.51</v>
       </c>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="b">
@@ -3818,71 +3738,69 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr"/>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>REC Ltd</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>13.34</v>
+      </c>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" t="b">
+        <v>0</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
           <t>RELIANCE</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t xml:space="preserve">Reliance Industries Ltd
 </t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>Energy</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H76" t="n">
-        <v>9.609999999999999</v>
-      </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="b">
-        <v>0</v>
-      </c>
-      <c r="K76" t="b">
-        <v>0</v>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>SBILIFE</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>SBI Life Insurance Company Ltd</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Financials</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -3898,7 +3816,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>24.23</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="b">
@@ -3912,22 +3830,21 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SHREECEM</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Shree Cement Ltd</t>
+          <t>SBI Life Insurance Company Ltd</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -3943,7 +3860,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>10.33</v>
+        <v>24.23</v>
       </c>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="b">
@@ -3957,117 +3874,108 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>State Bank of India</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="b">
+        <v>0</v>
+      </c>
+      <c r="K79" t="b">
+        <v>0</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Shree Cement Ltd</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="b">
+        <v>0</v>
+      </c>
+      <c r="K80" t="b">
+        <v>0</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
           <t>SHRIRAMFIN</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t xml:space="preserve">Shriram Finance Ltd
 </t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>Financials</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H79" t="n">
-        <v>18.56</v>
-      </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="b">
-        <v>0</v>
-      </c>
-      <c r="K79" t="b">
-        <v>0</v>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>Growth Funded by Debt</t>
-        </is>
-      </c>
-      <c r="M79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>SIEMENS</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Siemens Ltd</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H80" t="n">
-        <v>11.19</v>
-      </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="b">
-        <v>0</v>
-      </c>
-      <c r="K80" t="b">
-        <v>0</v>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Sun Pharmaceuticals Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -4083,7 +3991,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>10.78</v>
+        <v>18.56</v>
       </c>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="b">
@@ -4094,25 +4002,24 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M81" t="inlineStr"/>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Tata Consumer Products Ltd</t>
+          <t>Siemens Ltd</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -4128,7 +4035,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>15.96</v>
+        <v>11.19</v>
       </c>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="b">
@@ -4139,25 +4046,24 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Mixed</t>
-        </is>
-      </c>
-      <c r="M82" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Tata Motors Ltd</t>
+          <t>Sun Pharmaceuticals Industries Ltd</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
@@ -4173,7 +4079,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>7.72</v>
+        <v>10.78</v>
       </c>
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="b">
@@ -4187,159 +4093,155 @@
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Tata Consumer Products Ltd</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>15.96</v>
+      </c>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="b">
+        <v>0</v>
+      </c>
+      <c r="K84" t="b">
+        <v>0</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>TATAMOTORS</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Tata Motors Ltd</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="b">
+        <v>0</v>
+      </c>
+      <c r="K85" t="b">
+        <v>0</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
           <t>TATAPOWER</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t xml:space="preserve">Tata Power Company Ltd
 </t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H84" t="n">
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
         <v>15.51</v>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="b">
-        <v>0</v>
-      </c>
-      <c r="K84" t="b">
-        <v>0</v>
-      </c>
-      <c r="L84" t="inlineStr">
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="b">
+        <v>0</v>
+      </c>
+      <c r="K86" t="b">
+        <v>0</v>
+      </c>
+      <c r="L86" t="inlineStr">
         <is>
           <t>Shareholder Returns</t>
         </is>
       </c>
-      <c r="M84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>TATASTEEL</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t xml:space="preserve">Tata Steel Ltd
 </t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Materials</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H85" t="n">
-        <v>7.77</v>
-      </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="b">
-        <v>0</v>
-      </c>
-      <c r="K85" t="b">
-        <v>0</v>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>TCS</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Tata Consultancy Services Ltd</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H86" t="n">
-        <v>10.46</v>
-      </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="b">
-        <v>0</v>
-      </c>
-      <c r="K86" t="b">
-        <v>0</v>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>Liquidating Assets</t>
-        </is>
-      </c>
-      <c r="M86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>TECHM</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Tech Mahindra Ltd</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
@@ -4355,7 +4257,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>8.4</v>
+        <v>7.77</v>
       </c>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="b">
@@ -4366,113 +4268,110 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr"/>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Ltd</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="b">
+        <v>0</v>
+      </c>
+      <c r="K88" t="b">
+        <v>0</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Tech Mahindra Ltd</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Information Technology</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="b">
+        <v>0</v>
+      </c>
+      <c r="K89" t="b">
+        <v>0</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
           <t>TITAN</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t xml:space="preserve">Titan Company Ltd
 </t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H88" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="b">
-        <v>0</v>
-      </c>
-      <c r="K88" t="b">
-        <v>0</v>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>Reinvestor</t>
-        </is>
-      </c>
-      <c r="M88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>TORNTPHARM</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Torrent Pharmaceuticals Ltd</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
-      </c>
-      <c r="H89" t="n">
-        <v>6.93</v>
-      </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="b">
-        <v>0</v>
-      </c>
-      <c r="K89" t="b">
-        <v>0</v>
-      </c>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t>Shareholder Returns</t>
-        </is>
-      </c>
-      <c r="M89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>TRENT</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Trent Ltd</t>
-        </is>
-      </c>
       <c r="C90" t="inlineStr">
         <is>
           <t>Consumer Discretionary</t>
@@ -4491,7 +4390,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>36.31</v>
+        <v>20.9</v>
       </c>
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="b">
@@ -4505,22 +4404,21 @@
           <t>Reinvestor</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TVSMOTOR</t>
+          <t>TORNTPHARM</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>TVS Motor Company Ltd</t>
+          <t>Torrent Pharmaceuticals Ltd</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
@@ -4536,7 +4434,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>14.19</v>
+        <v>6.93</v>
       </c>
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="b">
@@ -4547,10 +4445,97 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Trent Ltd</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
+        <v>36.31</v>
+      </c>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="b">
+        <v>0</v>
+      </c>
+      <c r="K92" t="b">
+        <v>0</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>TVS Motor Company Ltd</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Insufficient Data</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>14.19</v>
+      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="b">
+        <v>0</v>
+      </c>
+      <c r="K93" t="b">
+        <v>0</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
           <t>Growth Funded by Debt</t>
         </is>
       </c>
-      <c r="M91" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>